<commit_message>
Finalise V16 TAD (renamed to V16-Final) and workbook resave
- TADUnifiedMaritimePlatform-V16-Final.docx: the executive-register TAD,
  finalised in Word (renamed from V16-Executive, author edits applied) —
  142 pages, all screenshots and rebuilt figures intact.
- CommercialModel-V1.xlsx: resaved; totals still reconcile to 5,400,000.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/rfp-response/CommercialModel-V1.xlsx
+++ b/rfp-response/CommercialModel-V1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ashish/Claude/Projects/maritime-project-presentation/rfp-response/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3248BD85-85E7-1F48-8D10-52CD90531755}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42A82D51-8201-304C-BF8A-CA7FB7B895ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20" yWindow="600" windowWidth="27040" windowHeight="15800" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="20" yWindow="600" windowWidth="27040" windowHeight="15760" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="6" r:id="rId1"/>

</xml_diff>